<commit_message>
v4 Phase 3: wire portfolio_boards.py into discover.py, add eligibility filtering
</commit_message>
<xml_diff>
--- a/results/joey/LATAM/Week_of_2026-07-20/Scored_LATAM_Joey_Complete_2026-07-20.xlsx
+++ b/results/joey/LATAM/Week_of_2026-07-20/Scored_LATAM_Joey_Complete_2026-07-20.xlsx
@@ -820,7 +820,7 @@
         <v>0</v>
       </c>
       <c r="AB2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
@@ -834,11 +834,15 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>Director-level payer GTM operations role in US value-based care, a healthcare-specific domain outside Joey's fintech/VC/government background, and the posting is listed simply as "Remote, United States" with no LATAM or international-candidate language.</t>
+          <t>Director-level GTM/operations role has real structural overlap with Joey's cross-functional program work, but it is healthcare-payer domain-gated (value-based care, ACOs, Medicare Advantage) with no LATAM signal. Location is explicitly "Remote, United States," a hard geographic disqualifier.</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Domain, Geography</t>
+        </is>
+      </c>
       <c r="AH2" t="inlineStr">
         <is>
           <t>not_mentioned</t>
@@ -870,16 +874,16 @@
         </is>
       </c>
       <c r="AN2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AO2" t="n">
         <v>0</v>
       </c>
       <c r="AP2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AQ2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -1013,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="AB3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
@@ -1027,11 +1031,15 @@
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>This is an individual-contributor GTM systems-builder/CSM role at the 4+ year level, not a Director/VP-caliber strategy or partnerships position, and it is posted as "Remote, United States" with pay tiers scoped to US locations only.</t>
+          <t>This is an individual-contributor "GTM Engineer" role (4+ years, book-of-accounts CSM/RevOps hybrid), well below Joey's Director/SVP calibration and outside his sector focus. Location is "Remote, United States" with no LATAM mention, a hard disqualifier.</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Function, Level, Geography</t>
+        </is>
+      </c>
       <c r="AH3" t="inlineStr">
         <is>
           <t>not_mentioned</t>
@@ -1044,7 +1052,7 @@
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>130000-165000</t>
+          <t>$130,000-$165,000</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
@@ -1069,10 +1077,10 @@
         <v>0</v>
       </c>
       <c r="AP3" t="n">
+        <v>8</v>
+      </c>
+      <c r="AQ3" t="n">
         <v>6</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1206,7 +1214,7 @@
         <v>0</v>
       </c>
       <c r="AB4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
@@ -1220,11 +1228,15 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>Despite executive-facing multithreading responsibilities, this is a 6+ year individual-contributor account role rather than a Director+ position, and the listing is "Remote, United States" with pay tiers explicitly scoped to US locations.</t>
+          <t>Mid-Market GTM Engineer is a senior IC account-management role (6+ years) requiring "3+ stakeholders per account" multithreading, not a Director-level strategy or CoS mandate. Location is "Remote, United States," a hard geographic disqualifier with no LATAM scope stated.</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Function, Level, Geography</t>
+        </is>
+      </c>
       <c r="AH4" t="inlineStr">
         <is>
           <t>not_mentioned</t>
@@ -1237,7 +1249,7 @@
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>150000-175000</t>
+          <t>$150,000-$175,000</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
@@ -1256,16 +1268,16 @@
         </is>
       </c>
       <c r="AN4" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="AO4" t="n">
         <v>0</v>
       </c>
       <c r="AP4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AQ4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -1399,7 +1411,7 @@
         <v>0</v>
       </c>
       <c r="AB5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
@@ -1413,11 +1425,15 @@
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>The Head of Growth Marketing scope and executive exposure are a reasonable operator fit, but the JD states candidates "must be legally authorized to work in the United States" even under the "Remote (Americas)" option, which contradicts genuine LATAM openness.</t>
+          <t>"Remote (Americas, UTC-3 to UTC-10)" reads LATAM-open, but the JD states candidates "must be legally authorized to work in the United States" with no sponsorship, which is a US-residency disqualifier regardless of the timezone framing. The role itself is also a hands-on growth-marketing/channel-ops seat (SEO, content, paid channels), a domain and function stretch from Joey's CoS/BizOps/partnerships background.</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>Domain, Function, Geography</t>
+        </is>
+      </c>
       <c r="AH5" t="inlineStr">
         <is>
           <t>not_mentioned</t>
@@ -1430,7 +1446,7 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>200000-250000</t>
+          <t>$200,000-$250,000</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
@@ -1440,7 +1456,7 @@
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>Eric</t>
+          <t>Eric (growth strategy owner) - no formal title given</t>
         </is>
       </c>
       <c r="AM5" t="inlineStr">
@@ -1449,13 +1465,13 @@
         </is>
       </c>
       <c r="AN5" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="AO5" t="n">
         <v>0</v>
       </c>
       <c r="AP5" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AQ5" t="n">
         <v>7</v>
@@ -1592,7 +1608,7 @@
         <v>0</v>
       </c>
       <c r="AB6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
@@ -1606,11 +1622,15 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Strong program-management/cross-functional skills match, but the listing is titled "Remote, Bangalore" and requires applicants to confirm they are currently based in Bangalore, with no LATAM or open-remote signal.</t>
+          <t>The cross-functional program-management scope (IT/Finance/Legal stakeholders, governance frameworks) echoes Joey's DoD program-management background reasonably well, but the posting is anchored to a specific non-LATAM city, asking "Are you currently based in Bangalore?" This is a hard geographic disqualifier with zero LATAM relevance in the enterprise DevSecOps/IT domain.</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>Domain, Geography</t>
+        </is>
+      </c>
       <c r="AH6" t="inlineStr">
         <is>
           <t>not_mentioned</t>
@@ -1642,7 +1662,7 @@
         </is>
       </c>
       <c r="AN6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -1651,7 +1671,7 @@
         <v>15</v>
       </c>
       <c r="AQ6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -1799,15 +1819,11 @@
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>Location is stated as "Remote, US" with no LATAM signal, and the role is a Finance-native transformation mandate (SOX, Lead-to-Cash, billing architecture) outside Joey's BD/CoS background. Disqualified on geography.</t>
+          <t>Explicitly listed as "Remote, US" with no international-candidate language, so this is a US work-location role outside LATAM scope. It is also a Finance-domain-owned VP role (SOX, revenue recognition, Lead-to-Cash) rather than a general CoS/ops/partnerships mandate.</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>Domain, Geography</t>
-        </is>
-      </c>
+      <c r="AG7" t="inlineStr"/>
       <c r="AH7" t="inlineStr">
         <is>
           <t>not_mentioned</t>
@@ -1825,7 +1841,7 @@
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>us_level</t>
+          <t>unclear</t>
         </is>
       </c>
       <c r="AL7" t="inlineStr">
@@ -1835,7 +1851,7 @@
       </c>
       <c r="AM7" t="inlineStr">
         <is>
-          <t>zero_to_one</t>
+          <t>scale_existing</t>
         </is>
       </c>
       <c r="AN7" t="n">
@@ -1845,10 +1861,10 @@
         <v>0</v>
       </c>
       <c r="AP7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AQ7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -1996,15 +2012,11 @@
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>Explicitly "Remote, United States" with E-Verify/I-9 language confirming US-only hiring, and the role is a hands-on technical GTM engineering IC job (Clay/Claude workflow-building) unrelated to Joey's strategic operator background. Disqualified on geography.</t>
+          <t>Location is stated as "Remote, United States" with an E-Verify/I-9 requirement, placing it outside LATAM scope. The role itself is a hands-on technical GTM engineering IC position (Clay, APIs, prompt workflows), not a CoS/Country Manager/senior BD match.</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>Function, Domain, Geography</t>
-        </is>
-      </c>
+      <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="inlineStr">
         <is>
           <t>not_mentioned</t>
@@ -2017,7 +2029,7 @@
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>130000-180000</t>
+          <t>$130,000 - $180,000 USD per year</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
@@ -2042,7 +2054,7 @@
         <v>0</v>
       </c>
       <c r="AP8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AQ8" t="n">
         <v>5</v>
@@ -2193,15 +2205,11 @@
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Listed as "Remote" but salary bands are scoped entirely to US labor-cost zones (Zone A-C cities) with Zone D explicitly unfunded, indicating a US-only hire; the role is also a Manager-level enablement/training function reporting to a Director, below Joey's target seniority. Disqualified on geography.</t>
+          <t>Salary band is scoped to US geographic zones ("Zones A-C"), indicating a US work location despite the bare "Remote" location string. Seniority sits below Director as an individual GTM Enablement Manager, and the function (training/enablement content) is a partial match at best to Joey's CoS/partnerships/ops background.</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>Function, Level, Geography</t>
-        </is>
-      </c>
+      <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr">
         <is>
           <t>not_mentioned</t>
@@ -2214,7 +2222,7 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>108650-142224</t>
+          <t>$108,650.00 - $142,224.00</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
@@ -2233,7 +2241,7 @@
         </is>
       </c>
       <c r="AN9" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AO9" t="n">
         <v>0</v>
@@ -2390,15 +2398,11 @@
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>Role is bound to "Remote, UK" and requires personally building the EMEA region hands-on with no LATAM scope stated; sector is ad-tech/performance marketing, listed as a poor fit under the rubric. Disqualified on geography.</t>
+          <t>Role is explicitly scoped to "Remote, UK" / EMEA with country-of-residence and work-authorization screening questions, entirely outside LATAM geography. It also requires a specific must-have background "building out EMEA for an ad-tech company," a domain Joey hasn't worked in.</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>Geography</t>
-        </is>
-      </c>
+      <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="inlineStr">
         <is>
           <t>not_mentioned</t>
@@ -2430,13 +2434,13 @@
         </is>
       </c>
       <c r="AN10" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="AO10" t="n">
         <v>0</v>
       </c>
       <c r="AP10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="AQ10" t="n">
         <v>5</v>
@@ -2587,15 +2591,11 @@
       </c>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>Location is "Remote - NY" and the JD requires work authorization in the US without sponsorship, with no LATAM signal; the individual-contributor Manager scope (4-6 years experience framing) also sits below Joey's target seniority. Disqualified on geography.</t>
+          <t>JD states candidates "must be authorized to work in the United States without... sponsorship," confirming a US-only work location. The role is also explicitly an individual-contributor position requiring hospital-RCM/IDR domain SME and SQL/BigQuery fluency, a significant domain and technical gap from Joey's background.</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="inlineStr">
-        <is>
-          <t>Level, Geography</t>
-        </is>
-      </c>
+      <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr">
         <is>
           <t>not_mentioned</t>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>120000-150000</t>
+          <t>$120K - $150K</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr">
@@ -2627,7 +2627,7 @@
         </is>
       </c>
       <c r="AN11" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="AO11" t="n">
         <v>0</v>
@@ -2636,7 +2636,7 @@
         <v>10</v>
       </c>
       <c r="AQ11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -2784,13 +2784,13 @@
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>Role is restricted to 'Remote - DACH' with deep German payroll/DATEV requirements, giving no LATAM signal despite Remote.com's EOR/cross-border sector fit. It is also a payroll-implementation specialist track reporting to a Payroll Operations manager, not a CoS/BD/strategy function.</t>
+          <t>Role is restricted to 'Remote - DACH,' a specific non-LATAM regional lock with no stated LATAM openness. It is also a payroll-implementation specialist function (DATEV expertise, German legislative knowledge) rather than the CoS/BD/strategic-ops work Joey targets.</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>Function, Level</t>
+          <t>function, domain</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>$77,600-$87,300 (converted from EUR71,850-EUR80,800)</t>
+          <t>approx $77,600-$87,300 (from €71,850-€80,800 EUR)</t>
         </is>
       </c>
       <c r="AK12" t="inlineStr">
@@ -2981,13 +2981,13 @@
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>Rula states it hires in 'most U.S. states' with no LATAM or international remote option, and the role is a SQL-heavy provider-quality Manager position rather than an executive-facing strategy/BD mandate. Sector (mental healthcare) also carries no stated LATAM relevance.</t>
+          <t>JD explicitly states the company hires only within the U.S. ('must be based in United States, currently not hiring in Hawaii'), which is a hard geo_restricted disqualifier regardless of fit. Underlying function (strategy &amp; ops, data-driven programs) is a partial skills match but the mental-healthcare sector isn't among Joey's priority verticals.</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>Function, Domain, Level</t>
+          <t>geography</t>
         </is>
       </c>
       <c r="AH13" t="inlineStr">
@@ -3027,10 +3027,10 @@
         <v>0</v>
       </c>
       <c r="AP13" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="AQ13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -3178,13 +3178,13 @@
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>Upwork states it hires full-time employees in only '34 U.S. states' with a Palo Alto home base, giving no LATAM or open-remote signal despite a strong Sr Director-level strategy/BD fit. The role's core function is hands-on M&amp;A sourcing and integration execution, a step beyond Joey's partnerships/financing-deal background.</t>
+          <t>JD asks for current/planned U.S. state of residence and the company hires full-time only across 34 U.S. states, a geo_restricted disqualifier with no LATAM or international remote path stated. Sr. Director-level scope and executive exposure fit Joey's seniority, but hands-on M&amp;A/corp-dev deal execution is a domain stretch beyond his banking and partnerships background.</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>Function, Geography</t>
+          <t>domain, geography</t>
         </is>
       </c>
       <c r="AH14" t="inlineStr">
@@ -3218,7 +3218,7 @@
         </is>
       </c>
       <c r="AN14" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="AO14" t="n">
         <v>0</v>
@@ -3227,7 +3227,7 @@
         <v>19</v>
       </c>
       <c r="AQ14" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>